<commit_message>
data(columns): reorder all Clean files to the v2 template, sync codebooks and clean scripts
- 45 *_Clean.csv reordered to the SKILL v2 template (Task right after
  Subject/[Group]/[Session]; Matching before Shape; Shape/Label identity
  triples adjacent to their parent column; study-specific extras kept at the tail)
- codebook row orders synced to the new column order (contents unchanged
  apart from HTML-entity normalisation)
- 11 clean scripts updated so a re-run reproduces the reordered files, each
  with a stopifnot(identical(names(...), c(...))) column-order guard
- verification: reordered files compared cell-by-cell with the previous
  revision (column set identical, no value changed); every script re-run and
  compared value-level against the working-tree file (0 differing cells)
</commit_message>
<xml_diff>
--- a/1_Data/Liang_2022_HumBrainMap/Codebook_Liang_2022_HumBrainMap_Exp1_Clean.xlsx
+++ b/1_Data/Liang_2022_HumBrainMap/Codebook_Liang_2022_HumBrainMap_Exp1_Clean.xlsx
@@ -50,6 +50,15 @@
     <t xml:space="preserve">Categorical</t>
   </si>
   <si>
+    <t xml:space="preserve">Task</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Task type: self-matching (shape-label matching with self/friend/stranger associations)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">self-matching</t>
+  </si>
+  <si>
     <t xml:space="preserve">Phase</t>
   </si>
   <si>
@@ -59,6 +68,15 @@
     <t xml:space="preserve">post;pre</t>
   </si>
   <si>
+    <t xml:space="preserve">Matching</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Whether the presented shape-label pair matches the learned association</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nonmatching;Matching</t>
+  </si>
+  <si>
     <t xml:space="preserve">Shape</t>
   </si>
   <si>
@@ -66,24 +84,6 @@
   </si>
   <si>
     <t xml:space="preserve">stranger;self;friend</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Task</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Task type: self-matching (shape-label matching with self/friend/stranger associations)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">self-matching</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Matching</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Whether the presented shape-label pair matches the learned association</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nonmatching;Matching</t>
   </si>
   <si>
     <t xml:space="preserve">Shape_Origin_Identity</t>

</xml_diff>